<commit_message>
Se agrega costos empleados
</commit_message>
<xml_diff>
--- a/trimestre 2/Lista de costos.xlsx
+++ b/trimestre 2/Lista de costos.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aprendiz\Desktop\Nueva carpeta\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aprendiz\Desktop\XD\RoyalPets\trimestre 2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{88B0134B-3763-420F-A46D-87537490C648}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6507BA69-FA49-4EAF-8FD2-C74E6B4C524A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CE73354B-E448-4686-BDAE-33FB59E1EA3A}"/>
   </bookViews>
@@ -68,9 +68,6 @@
     <t>Rol</t>
   </si>
   <si>
-    <t>Fase principal</t>
-  </si>
-  <si>
     <t>Horas estimadas</t>
   </si>
   <si>
@@ -210,6 +207,9 @@
   </si>
   <si>
     <t>Prestaciones tester.</t>
+  </si>
+  <si>
+    <t>Fase principal.</t>
   </si>
 </sst>
 </file>
@@ -219,7 +219,7 @@
   <numFmts count="3">
     <numFmt numFmtId="6" formatCode="&quot;$&quot;\ #,##0;[Red]\-&quot;$&quot;\ #,##0"/>
     <numFmt numFmtId="44" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="168" formatCode="_-[$$-240A]\ * #,##0.00_-;\-[$$-240A]\ * #,##0.00_-;_-[$$-240A]\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-[$$-240A]\ * #,##0.00_-;\-[$$-240A]\ * #,##0.00_-;_-[$$-240A]\ * &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -395,11 +395,11 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
@@ -411,9 +411,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -426,28 +423,31 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Moneda" xfId="1" builtinId="4"/>
@@ -803,19 +803,19 @@
         <v>8</v>
       </c>
       <c r="C2" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="D2" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="20" t="s">
+      <c r="E2" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="29" t="s">
+      <c r="F2" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="G2" s="20" t="s">
         <v>12</v>
-      </c>
-      <c r="G2" s="20" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.25">
@@ -826,10 +826,10 @@
         <v>4</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E3" s="16" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F3" s="17">
         <v>16800</v>
@@ -846,10 +846,10 @@
         <v>5</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F4" s="17">
         <v>27700</v>
@@ -866,10 +866,10 @@
         <v>6</v>
       </c>
       <c r="D5" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="E5" s="9" t="s">
         <v>39</v>
-      </c>
-      <c r="E5" s="9" t="s">
-        <v>40</v>
       </c>
       <c r="F5" s="17">
         <v>34600</v>
@@ -886,10 +886,10 @@
         <v>7</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F6" s="17">
         <v>17800</v>
@@ -899,662 +899,662 @@
       </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B8" s="23" t="s">
-        <v>43</v>
-      </c>
-      <c r="C8" s="23"/>
-      <c r="D8" s="23"/>
-      <c r="F8" s="23" t="s">
+      <c r="B8" s="36" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" s="36"/>
+      <c r="D8" s="36"/>
+      <c r="F8" s="36" t="s">
+        <v>50</v>
+      </c>
+      <c r="G8" s="36"/>
+      <c r="H8" s="36"/>
+      <c r="J8" s="37" t="s">
+        <v>16</v>
+      </c>
+      <c r="K8" s="37"/>
+      <c r="L8" s="37"/>
+    </row>
+    <row r="9" spans="2:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="B9" s="23" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" s="24" t="s">
         <v>51</v>
       </c>
-      <c r="G8" s="23"/>
-      <c r="H8" s="23"/>
-      <c r="J8" s="30" t="s">
+      <c r="D9" s="23" t="s">
+        <v>52</v>
+      </c>
+      <c r="F9" s="23" t="s">
+        <v>42</v>
+      </c>
+      <c r="G9" s="24" t="s">
+        <v>51</v>
+      </c>
+      <c r="H9" s="23" t="s">
+        <v>52</v>
+      </c>
+      <c r="J9" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="K8" s="30"/>
-      <c r="L8" s="30"/>
-    </row>
-    <row r="9" spans="2:12" ht="30" x14ac:dyDescent="0.25">
-      <c r="B9" s="24" t="s">
-        <v>43</v>
-      </c>
-      <c r="C9" s="25" t="s">
-        <v>52</v>
-      </c>
-      <c r="D9" s="24" t="s">
-        <v>53</v>
-      </c>
-      <c r="F9" s="24" t="s">
-        <v>43</v>
-      </c>
-      <c r="G9" s="25" t="s">
-        <v>52</v>
-      </c>
-      <c r="H9" s="24" t="s">
-        <v>53</v>
-      </c>
-      <c r="J9" s="2" t="s">
-        <v>18</v>
-      </c>
       <c r="K9" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B10" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="29" t="s">
         <v>25</v>
-      </c>
-      <c r="L9" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B10" s="26" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" s="31" t="s">
-        <v>26</v>
       </c>
       <c r="D10" s="15">
         <v>144500</v>
       </c>
-      <c r="F10" s="26" t="s">
-        <v>14</v>
-      </c>
-      <c r="G10" s="31" t="s">
-        <v>26</v>
-      </c>
-      <c r="H10" s="35">
+      <c r="F10" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10" s="29" t="s">
+        <v>25</v>
+      </c>
+      <c r="H10" s="33">
         <v>238000</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="L10" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B11" s="26" t="s">
-        <v>44</v>
-      </c>
-      <c r="C11" s="32">
+      <c r="B11" s="25" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" s="30">
         <v>0.12</v>
       </c>
       <c r="D11" s="15">
         <v>204000</v>
       </c>
-      <c r="F11" s="26" t="s">
-        <v>44</v>
-      </c>
-      <c r="G11" s="32">
+      <c r="F11" s="25" t="s">
+        <v>43</v>
+      </c>
+      <c r="G11" s="30">
         <v>0.12</v>
       </c>
-      <c r="H11" s="36">
+      <c r="H11" s="34">
         <v>336000</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="K11" s="7">
         <v>0.12</v>
       </c>
       <c r="L11" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12" spans="2:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="26" t="s">
-        <v>45</v>
-      </c>
-      <c r="C12" s="33" t="s">
-        <v>27</v>
+      <c r="B12" s="25" t="s">
+        <v>44</v>
+      </c>
+      <c r="C12" s="31" t="s">
+        <v>26</v>
       </c>
       <c r="D12" s="15">
         <v>118320</v>
       </c>
-      <c r="F12" s="26" t="s">
+      <c r="F12" s="25" t="s">
+        <v>44</v>
+      </c>
+      <c r="G12" s="31" t="s">
+        <v>26</v>
+      </c>
+      <c r="H12" s="34">
+        <v>194880</v>
+      </c>
+      <c r="J12" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="K12" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="L12" s="6" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="2:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="B13" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="G12" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="H12" s="36">
-        <v>194880</v>
-      </c>
-      <c r="J12" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="K12" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="L12" s="6" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="13" spans="2:12" ht="45" x14ac:dyDescent="0.25">
-      <c r="B13" s="27" t="s">
-        <v>46</v>
-      </c>
-      <c r="C13" s="34">
+      <c r="C13" s="32">
         <v>0.04</v>
       </c>
       <c r="D13" s="15">
         <v>68000</v>
       </c>
-      <c r="F13" s="27" t="s">
-        <v>46</v>
-      </c>
-      <c r="G13" s="34">
+      <c r="F13" s="26" t="s">
+        <v>45</v>
+      </c>
+      <c r="G13" s="32">
         <v>0.04</v>
       </c>
-      <c r="H13" s="35">
+      <c r="H13" s="33">
         <v>112000</v>
       </c>
       <c r="J13" s="8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K13" s="7">
         <v>0.04</v>
       </c>
       <c r="L13" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B14" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="C14" s="32">
+      <c r="B14" s="25" t="s">
+        <v>19</v>
+      </c>
+      <c r="C14" s="30">
         <v>0.02</v>
       </c>
       <c r="D14" s="15">
         <v>34000</v>
       </c>
-      <c r="F14" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="G14" s="32">
+      <c r="F14" s="25" t="s">
+        <v>19</v>
+      </c>
+      <c r="G14" s="30">
         <v>0.02</v>
       </c>
-      <c r="H14" s="35">
+      <c r="H14" s="33">
         <v>56000</v>
       </c>
       <c r="J14" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K14" s="7">
         <v>0.02</v>
       </c>
       <c r="L14" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B15" s="26" t="s">
-        <v>21</v>
-      </c>
-      <c r="C15" s="32">
+      <c r="B15" s="25" t="s">
+        <v>20</v>
+      </c>
+      <c r="C15" s="30">
         <v>0.03</v>
       </c>
       <c r="D15" s="15">
         <v>51000</v>
       </c>
-      <c r="F15" s="26" t="s">
-        <v>21</v>
-      </c>
-      <c r="G15" s="32">
+      <c r="F15" s="25" t="s">
+        <v>20</v>
+      </c>
+      <c r="G15" s="30">
         <v>0.03</v>
       </c>
-      <c r="H15" s="35">
+      <c r="H15" s="33">
         <v>84000</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K15" s="7">
         <v>0.03</v>
       </c>
       <c r="L15" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="16" spans="2:12" ht="30" x14ac:dyDescent="0.25">
-      <c r="B16" s="26" t="s">
-        <v>47</v>
-      </c>
-      <c r="C16" s="31" t="s">
-        <v>28</v>
+      <c r="B16" s="25" t="s">
+        <v>46</v>
+      </c>
+      <c r="C16" s="29" t="s">
+        <v>27</v>
       </c>
       <c r="D16" s="15">
         <v>141610</v>
       </c>
-      <c r="F16" s="26" t="s">
+      <c r="F16" s="25" t="s">
+        <v>46</v>
+      </c>
+      <c r="G16" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="H16" s="33">
+        <v>233240</v>
+      </c>
+      <c r="J16" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K16" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="L16" s="6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B17" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="G16" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="H16" s="35">
-        <v>233240</v>
-      </c>
-      <c r="J16" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="K16" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="L16" s="6" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B17" s="26" t="s">
-        <v>48</v>
-      </c>
-      <c r="C17" s="31" t="s">
-        <v>28</v>
+      <c r="C17" s="29" t="s">
+        <v>27</v>
       </c>
       <c r="D17" s="15">
         <v>141610</v>
       </c>
-      <c r="F17" s="26" t="s">
+      <c r="F17" s="25" t="s">
+        <v>47</v>
+      </c>
+      <c r="G17" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="H17" s="33">
+        <v>233240</v>
+      </c>
+      <c r="J17" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K17" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="L17" s="6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="18" spans="2:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="B18" s="26" t="s">
         <v>48</v>
       </c>
-      <c r="G17" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="H17" s="35">
-        <v>233240</v>
-      </c>
-      <c r="J17" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="K17" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="L17" s="6" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="18" spans="2:12" ht="45" x14ac:dyDescent="0.25">
-      <c r="B18" s="27" t="s">
-        <v>49</v>
-      </c>
-      <c r="C18" s="32">
+      <c r="C18" s="30">
         <v>0.01</v>
       </c>
       <c r="D18" s="15">
         <v>17000</v>
       </c>
-      <c r="F18" s="27" t="s">
-        <v>49</v>
-      </c>
-      <c r="G18" s="32">
+      <c r="F18" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="G18" s="30">
         <v>0.01</v>
       </c>
-      <c r="H18" s="35">
+      <c r="H18" s="33">
         <v>28000</v>
       </c>
       <c r="J18" s="8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K18" s="7">
         <v>0.01</v>
       </c>
       <c r="L18" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="19" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B19" s="26" t="s">
+      <c r="B19" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="C19" s="29" t="s">
         <v>29</v>
-      </c>
-      <c r="C19" s="31" t="s">
-        <v>30</v>
       </c>
       <c r="D19" s="15">
         <v>70890</v>
       </c>
-      <c r="F19" s="26" t="s">
+      <c r="F19" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="G19" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="G19" s="31" t="s">
-        <v>30</v>
-      </c>
-      <c r="H19" s="35">
+      <c r="H19" s="33">
         <v>116760</v>
       </c>
       <c r="J19" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="K19" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="K19" s="5" t="s">
-        <v>30</v>
-      </c>
       <c r="L19" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B20" s="28" t="s">
-        <v>50</v>
-      </c>
-      <c r="C20" s="31" t="s">
-        <v>54</v>
+      <c r="B20" s="27" t="s">
+        <v>49</v>
+      </c>
+      <c r="C20" s="29" t="s">
+        <v>53</v>
       </c>
       <c r="D20" s="15">
         <v>990930</v>
       </c>
-      <c r="F20" s="28" t="s">
-        <v>50</v>
-      </c>
-      <c r="G20" s="31" t="s">
+      <c r="F20" s="27" t="s">
+        <v>49</v>
+      </c>
+      <c r="G20" s="29" t="s">
+        <v>53</v>
+      </c>
+      <c r="H20" s="33">
+        <v>1632120</v>
+      </c>
+    </row>
+    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B23" s="36" t="s">
         <v>54</v>
       </c>
-      <c r="H20" s="35">
-        <v>1632120</v>
-      </c>
-    </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B23" s="23" t="s">
+      <c r="C23" s="36"/>
+      <c r="D23" s="36"/>
+      <c r="F23" s="36" t="s">
         <v>55</v>
       </c>
-      <c r="C23" s="23"/>
-      <c r="D23" s="23"/>
-      <c r="F23" s="23" t="s">
-        <v>56</v>
-      </c>
-      <c r="G23" s="23"/>
-      <c r="H23" s="23"/>
+      <c r="G23" s="36"/>
+      <c r="H23" s="36"/>
     </row>
     <row r="24" spans="2:12" ht="30" x14ac:dyDescent="0.25">
-      <c r="B24" s="24" t="s">
-        <v>43</v>
-      </c>
-      <c r="C24" s="25" t="s">
+      <c r="B24" s="23" t="s">
+        <v>42</v>
+      </c>
+      <c r="C24" s="24" t="s">
+        <v>51</v>
+      </c>
+      <c r="D24" s="24" t="s">
         <v>52</v>
       </c>
-      <c r="D24" s="25" t="s">
-        <v>53</v>
-      </c>
-      <c r="F24" s="24" t="s">
-        <v>43</v>
-      </c>
-      <c r="G24" s="25" t="s">
+      <c r="F24" s="23" t="s">
+        <v>42</v>
+      </c>
+      <c r="G24" s="24" t="s">
+        <v>51</v>
+      </c>
+      <c r="H24" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="H24" s="24" t="s">
-        <v>53</v>
-      </c>
     </row>
     <row r="25" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B25" s="26" t="s">
-        <v>14</v>
-      </c>
-      <c r="C25" s="31" t="s">
-        <v>26</v>
+      <c r="B25" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="C25" s="29" t="s">
+        <v>25</v>
       </c>
       <c r="D25" s="15">
         <v>297500</v>
       </c>
-      <c r="F25" s="26" t="s">
-        <v>14</v>
-      </c>
-      <c r="G25" s="31" t="s">
-        <v>26</v>
-      </c>
-      <c r="H25" s="37">
+      <c r="F25" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="G25" s="29" t="s">
+        <v>25</v>
+      </c>
+      <c r="H25" s="35">
         <v>153000</v>
       </c>
     </row>
     <row r="26" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B26" s="26" t="s">
-        <v>44</v>
-      </c>
-      <c r="C26" s="32">
+      <c r="B26" s="25" t="s">
+        <v>43</v>
+      </c>
+      <c r="C26" s="30">
         <v>0.12</v>
       </c>
       <c r="D26" s="15">
         <v>420000</v>
       </c>
-      <c r="F26" s="26" t="s">
+      <c r="F26" s="25" t="s">
+        <v>43</v>
+      </c>
+      <c r="G26" s="30">
+        <v>0.12</v>
+      </c>
+      <c r="H26" s="35">
+        <v>216000</v>
+      </c>
+    </row>
+    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B27" s="25" t="s">
         <v>44</v>
       </c>
-      <c r="G26" s="32">
-        <v>0.12</v>
-      </c>
-      <c r="H26" s="37">
-        <v>216000</v>
-      </c>
-    </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B27" s="26" t="s">
-        <v>45</v>
-      </c>
-      <c r="C27" s="33" t="s">
-        <v>27</v>
+      <c r="C27" s="31" t="s">
+        <v>26</v>
       </c>
       <c r="D27" s="15">
         <v>243600</v>
       </c>
-      <c r="F27" s="26" t="s">
+      <c r="F27" s="25" t="s">
+        <v>44</v>
+      </c>
+      <c r="G27" s="31" t="s">
+        <v>26</v>
+      </c>
+      <c r="H27" s="35">
+        <v>125280</v>
+      </c>
+    </row>
+    <row r="28" spans="2:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="B28" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="G27" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="H27" s="37">
-        <v>125280</v>
-      </c>
-    </row>
-    <row r="28" spans="2:12" ht="30" x14ac:dyDescent="0.25">
-      <c r="B28" s="27" t="s">
-        <v>46</v>
-      </c>
-      <c r="C28" s="34">
+      <c r="C28" s="32">
         <v>0.04</v>
       </c>
       <c r="D28" s="15">
         <v>140000</v>
       </c>
-      <c r="F28" s="27" t="s">
-        <v>46</v>
-      </c>
-      <c r="G28" s="34">
+      <c r="F28" s="26" t="s">
+        <v>45</v>
+      </c>
+      <c r="G28" s="32">
         <v>0.04</v>
       </c>
-      <c r="H28" s="37">
+      <c r="H28" s="35">
         <v>72000</v>
       </c>
     </row>
     <row r="29" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B29" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="C29" s="32">
+      <c r="B29" s="25" t="s">
+        <v>19</v>
+      </c>
+      <c r="C29" s="30">
         <v>0.02</v>
       </c>
       <c r="D29" s="15">
         <v>70000</v>
       </c>
-      <c r="F29" s="26" t="s">
+      <c r="F29" s="25" t="s">
+        <v>19</v>
+      </c>
+      <c r="G29" s="30">
+        <v>0.02</v>
+      </c>
+      <c r="H29" s="35">
+        <v>36000</v>
+      </c>
+    </row>
+    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B30" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="G29" s="32">
-        <v>0.02</v>
-      </c>
-      <c r="H29" s="37">
-        <v>36000</v>
-      </c>
-    </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B30" s="26" t="s">
-        <v>21</v>
-      </c>
-      <c r="C30" s="32">
+      <c r="C30" s="30">
         <v>0.03</v>
       </c>
       <c r="D30" s="15">
         <v>105000</v>
       </c>
-      <c r="F30" s="26" t="s">
-        <v>21</v>
-      </c>
-      <c r="G30" s="32">
+      <c r="F30" s="25" t="s">
+        <v>20</v>
+      </c>
+      <c r="G30" s="30">
         <v>0.03</v>
       </c>
-      <c r="H30" s="37">
+      <c r="H30" s="35">
         <v>54000</v>
       </c>
     </row>
     <row r="31" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B31" s="26" t="s">
-        <v>47</v>
-      </c>
-      <c r="C31" s="31" t="s">
-        <v>28</v>
+      <c r="B31" s="25" t="s">
+        <v>46</v>
+      </c>
+      <c r="C31" s="29" t="s">
+        <v>27</v>
       </c>
       <c r="D31" s="15">
         <v>291550</v>
       </c>
-      <c r="F31" s="26" t="s">
+      <c r="F31" s="25" t="s">
+        <v>46</v>
+      </c>
+      <c r="G31" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="H31" s="35">
+        <v>149940</v>
+      </c>
+    </row>
+    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B32" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="G31" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="H31" s="37">
-        <v>149940</v>
-      </c>
-    </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B32" s="26" t="s">
-        <v>48</v>
-      </c>
-      <c r="C32" s="31" t="s">
-        <v>28</v>
+      <c r="C32" s="29" t="s">
+        <v>27</v>
       </c>
       <c r="D32" s="15">
         <v>291550</v>
       </c>
-      <c r="F32" s="26" t="s">
+      <c r="F32" s="25" t="s">
+        <v>47</v>
+      </c>
+      <c r="G32" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="H32" s="35">
+        <v>149940</v>
+      </c>
+    </row>
+    <row r="33" spans="2:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="B33" s="26" t="s">
         <v>48</v>
       </c>
-      <c r="G32" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="H32" s="37">
-        <v>149940</v>
-      </c>
-    </row>
-    <row r="33" spans="2:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="B33" s="27" t="s">
-        <v>49</v>
-      </c>
-      <c r="C33" s="32">
+      <c r="C33" s="30">
         <v>0.01</v>
       </c>
       <c r="D33" s="15">
         <v>35000</v>
       </c>
-      <c r="F33" s="27" t="s">
-        <v>49</v>
-      </c>
-      <c r="G33" s="32">
+      <c r="F33" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="G33" s="30">
         <v>0.01</v>
       </c>
-      <c r="H33" s="37">
+      <c r="H33" s="35">
         <v>18000</v>
       </c>
     </row>
     <row r="34" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B34" s="26" t="s">
+      <c r="B34" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="C34" s="29" t="s">
         <v>29</v>
-      </c>
-      <c r="C34" s="31" t="s">
-        <v>30</v>
       </c>
       <c r="D34" s="15">
         <v>145950</v>
       </c>
-      <c r="F34" s="26" t="s">
+      <c r="F34" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="G34" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="G34" s="31" t="s">
-        <v>30</v>
-      </c>
-      <c r="H34" s="37">
+      <c r="H34" s="35">
         <v>75060</v>
       </c>
     </row>
     <row r="35" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B35" s="28"/>
-      <c r="C35" s="31" t="s">
-        <v>54</v>
+      <c r="B35" s="27"/>
+      <c r="C35" s="29" t="s">
+        <v>53</v>
       </c>
       <c r="D35" s="15">
         <v>2039150</v>
       </c>
-      <c r="F35" s="28"/>
-      <c r="G35" s="31" t="s">
-        <v>54</v>
-      </c>
-      <c r="H35" s="37">
+      <c r="F35" s="27"/>
+      <c r="G35" s="29" t="s">
+        <v>53</v>
+      </c>
+      <c r="H35" s="35">
         <v>1049220</v>
       </c>
     </row>
     <row r="46" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B46" s="18" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="47" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B47" s="18" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="48" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B48" s="18" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="49" spans="2:2" ht="30" x14ac:dyDescent="0.25">
       <c r="B49" s="19" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="50" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B50" s="18" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="51" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B51" s="18" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="52" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B52" s="18" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="53" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B53" s="18" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="54" spans="2:2" ht="30" x14ac:dyDescent="0.25">
       <c r="B54" s="19" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="55" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B55" s="18" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="56" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B56" s="18" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Se agregaron las fichas técnicas
</commit_message>
<xml_diff>
--- a/trimestre 2/Lista de costos.xlsx
+++ b/trimestre 2/Lista de costos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aprendiz\Desktop\XD\RoyalPets\trimestre 2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F2F0CA3-941E-47A8-91C3-042CFF8ABAAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7EB9861-F232-435C-B0C3-0047444EF0C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CE73354B-E448-4686-BDAE-33FB59E1EA3A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{CE73354B-E448-4686-BDAE-33FB59E1EA3A}"/>
   </bookViews>
   <sheets>
     <sheet name="Costos empleados" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="102">
   <si>
     <t>Analista</t>
   </si>
@@ -202,17 +202,162 @@
   </si>
   <si>
     <t xml:space="preserve">Desarrollador </t>
+  </si>
+  <si>
+    <t>Computador #1 -  "Mas potente"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Computador #2 </t>
+  </si>
+  <si>
+    <t>Computador #3 "Mas economico"</t>
+  </si>
+  <si>
+    <t>Componentes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Precio </t>
+  </si>
+  <si>
+    <t>Detalles</t>
+  </si>
+  <si>
+    <t>CPU</t>
+  </si>
+  <si>
+    <t>AMD Ryzen 7 7700X</t>
+  </si>
+  <si>
+    <t>Alto rendimiento multinúcleo para compilación y virtualización.</t>
+  </si>
+  <si>
+    <t>Excelente rendimiento para compilar código y ejecutar contenedores.</t>
+  </si>
+  <si>
+    <t>Intel Core i7‑13700F</t>
+  </si>
+  <si>
+    <t>Alto rendimiento para análisis de datos y pruebas simultáneas.</t>
+  </si>
+  <si>
+    <t>GPU</t>
+  </si>
+  <si>
+    <t>GIGABYTE GeForce RTX 4060 WINDFORCE OC 8GB</t>
+  </si>
+  <si>
+    <t>Acelera IA, cálculos paralelos y múltiples monitores.</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>RAM</t>
+  </si>
+  <si>
+    <t>Corsair Vengeance DDR5 32GB (2x16GB) 6000MHz</t>
+  </si>
+  <si>
+    <t>Mucha memoria para multitarea y contenedores.</t>
+  </si>
+  <si>
+    <t>Corsair Vengeance DDR5 32GB (2x16GB)</t>
+  </si>
+  <si>
+    <t>Memoria suficiente para multitarea y entornos de desarrollo.</t>
+  </si>
+  <si>
+    <t>Corsair Vengeance DDR5 32GB</t>
+  </si>
+  <si>
+    <t>Memoria suficiente para múltiples herramientas y navegadores.</t>
+  </si>
+  <si>
+    <t>SSD</t>
+  </si>
+  <si>
+    <t>Samsung 980 Pro 1TB NVMe</t>
+  </si>
+  <si>
+    <t>Lectura ultrarrápida para proyectos y bases de datos.</t>
+  </si>
+  <si>
+    <t>Alta velocidad para cargar proyectos y bases de datos.</t>
+  </si>
+  <si>
+    <t>Almacenamiento rápido para pruebas y manejo de datos.</t>
+  </si>
+  <si>
+    <t>Motherboard</t>
+  </si>
+  <si>
+    <t>Gigabyte B650 Eagle AX</t>
+  </si>
+  <si>
+    <t>Compatible con Ryzen 7000 y expansión moderna.</t>
+  </si>
+  <si>
+    <t>Soporte moderno y buena conectividad para expansión futura.</t>
+  </si>
+  <si>
+    <t>ASRock B650M‑HDV </t>
+  </si>
+  <si>
+    <t>Placa base económica con soporte para componentes modernos.</t>
+  </si>
+  <si>
+    <t>Fuente de pdr</t>
+  </si>
+  <si>
+    <t>Aerocool Dorado 750W 80+ Gold </t>
+  </si>
+  <si>
+    <t>Energía estable y eficiente para componentes potentes.</t>
+  </si>
+  <si>
+    <t>Aerocool Dorado 750W</t>
+  </si>
+  <si>
+    <t>Fuente eficiente y estable para el sistema.</t>
+  </si>
+  <si>
+    <t>Gamdias 750W Gold</t>
+  </si>
+  <si>
+    <t>Fuente eficiente para estabilidad del sistema.</t>
+  </si>
+  <si>
+    <t>Gabinete</t>
+  </si>
+  <si>
+    <t>Xtech XT‑GMR3 Deimos ATX</t>
+  </si>
+  <si>
+    <t>Buen flujo de aire y espacio para expansión.</t>
+  </si>
+  <si>
+    <t>Xtech XT‑GMR3 Deimos</t>
+  </si>
+  <si>
+    <t>Gabinete económico con buen flujo de aire.</t>
+  </si>
+  <si>
+    <t>Gabinete con ventilación adecuada y espacio para componentes.</t>
+  </si>
+  <si>
+    <t>TOTAL</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="4">
+  <numFmts count="5">
+    <numFmt numFmtId="6" formatCode="&quot;$&quot;\ #,##0;[Red]\-&quot;$&quot;\ #,##0"/>
     <numFmt numFmtId="44" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_-[$$-240A]\ * #,##0.00_-;\-[$$-240A]\ * #,##0.00_-;_-[$$-240A]\ * &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="167" formatCode="_-&quot;$&quot;\ * #,##0_-;\-&quot;$&quot;\ * #,##0_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="168" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="_-&quot;$&quot;\ * #,##0_-;\-&quot;$&quot;\ * #,##0_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -246,7 +391,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="18">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -301,8 +446,56 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -351,13 +544,50 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -423,52 +653,116 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="8" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="6" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="3" fillId="8" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -487,6 +781,59 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="AutoShape 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3C3E924F-BDCE-4750-9496-C3F5B5A6B33D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="933450" y="3067050"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -812,7 +1159,7 @@
     <col min="2" max="2" width="15.42578125" customWidth="1"/>
     <col min="3" max="3" width="30.42578125" customWidth="1"/>
     <col min="4" max="4" width="15.85546875" customWidth="1"/>
-    <col min="5" max="5" width="16.85546875" style="38" customWidth="1"/>
+    <col min="5" max="5" width="16.85546875" style="36" customWidth="1"/>
     <col min="6" max="6" width="20.85546875" customWidth="1"/>
     <col min="7" max="7" width="25.7109375" customWidth="1"/>
     <col min="8" max="8" width="14.42578125" customWidth="1"/>
@@ -831,7 +1178,7 @@
       <c r="D2" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="33" t="s">
+      <c r="E2" s="31" t="s">
         <v>10</v>
       </c>
       <c r="F2" s="17" t="s">
@@ -851,7 +1198,7 @@
       <c r="D3" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="E3" s="34">
+      <c r="E3" s="32">
         <v>3000000</v>
       </c>
       <c r="F3" s="13">
@@ -873,7 +1220,7 @@
       <c r="D4" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="E4" s="35">
+      <c r="E4" s="33">
         <v>2800000</v>
       </c>
       <c r="F4" s="13">
@@ -893,7 +1240,7 @@
       <c r="D5" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="E5" s="36">
+      <c r="E5" s="34">
         <v>3500000</v>
       </c>
       <c r="F5" s="13">
@@ -913,7 +1260,7 @@
       <c r="D6" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="E6" s="37">
+      <c r="E6" s="35">
         <v>1800000</v>
       </c>
       <c r="F6" s="13">
@@ -924,21 +1271,21 @@
       </c>
     </row>
     <row r="8" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B8" s="31" t="s">
+      <c r="B8" s="46" t="s">
         <v>38</v>
       </c>
-      <c r="C8" s="31"/>
-      <c r="D8" s="31"/>
-      <c r="P8" s="31" t="s">
+      <c r="C8" s="46"/>
+      <c r="D8" s="46"/>
+      <c r="P8" s="46" t="s">
         <v>46</v>
       </c>
-      <c r="Q8" s="31"/>
-      <c r="R8" s="31"/>
-      <c r="T8" s="32" t="s">
+      <c r="Q8" s="46"/>
+      <c r="R8" s="46"/>
+      <c r="T8" s="47" t="s">
         <v>16</v>
       </c>
-      <c r="U8" s="32"/>
-      <c r="V8" s="32"/>
+      <c r="U8" s="47"/>
+      <c r="V8" s="47"/>
     </row>
     <row r="9" spans="2:22" ht="30" x14ac:dyDescent="0.25">
       <c r="B9" s="19" t="s">
@@ -950,13 +1297,13 @@
       <c r="D9" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="E9" s="46" t="s">
+      <c r="E9" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="F9" s="46" t="s">
+      <c r="F9" s="44" t="s">
         <v>53</v>
       </c>
-      <c r="G9" s="46" t="s">
+      <c r="G9" s="44" t="s">
         <v>3</v>
       </c>
       <c r="P9" s="19" t="s">
@@ -982,29 +1329,29 @@
       <c r="B10" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="42">
+      <c r="C10" s="40">
         <v>8.5000000000000006E-2</v>
       </c>
-      <c r="D10" s="41">
+      <c r="D10" s="39">
         <f>E$3*C10</f>
         <v>255000.00000000003</v>
       </c>
-      <c r="E10" s="41">
+      <c r="E10" s="39">
         <f>E$4*C10</f>
         <v>238000.00000000003</v>
       </c>
-      <c r="F10" s="41">
+      <c r="F10" s="39">
         <f>E$5*C10</f>
         <v>297500</v>
       </c>
-      <c r="G10" s="41">
+      <c r="G10" s="39">
         <f>E$6*C10</f>
         <v>153000</v>
       </c>
       <c r="P10" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="Q10" s="40">
+      <c r="Q10" s="38">
         <v>8.5000000000000006E-2</v>
       </c>
       <c r="R10" s="28">
@@ -1025,22 +1372,22 @@
       <c r="B11" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="C11" s="43">
+      <c r="C11" s="41">
         <v>0.12</v>
       </c>
-      <c r="D11" s="41">
-        <f t="shared" ref="D11:E20" si="0">E$3*C11</f>
+      <c r="D11" s="39">
+        <f t="shared" ref="D11:D19" si="0">E$3*C11</f>
         <v>360000</v>
       </c>
-      <c r="E11" s="41">
-        <f t="shared" ref="E11:G19" si="1">E$4*C11</f>
+      <c r="E11" s="39">
+        <f t="shared" ref="E11:E19" si="1">E$4*C11</f>
         <v>336000</v>
       </c>
-      <c r="F11" s="41">
+      <c r="F11" s="39">
         <f t="shared" ref="F11:F19" si="2">E$5*C11</f>
         <v>420000</v>
       </c>
-      <c r="G11" s="41">
+      <c r="G11" s="39">
         <f t="shared" ref="G11:G19" si="3">E$6*C11</f>
         <v>216000</v>
       </c>
@@ -1067,29 +1414,29 @@
       <c r="B12" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="C12" s="39">
+      <c r="C12" s="37">
         <v>5.2199999999999998E-3</v>
       </c>
-      <c r="D12" s="41">
+      <c r="D12" s="39">
         <f t="shared" si="0"/>
         <v>15660</v>
       </c>
-      <c r="E12" s="41">
+      <c r="E12" s="39">
         <f t="shared" si="1"/>
         <v>14616</v>
       </c>
-      <c r="F12" s="41">
+      <c r="F12" s="39">
         <f t="shared" si="2"/>
         <v>18270</v>
       </c>
-      <c r="G12" s="41">
+      <c r="G12" s="39">
         <f t="shared" si="3"/>
         <v>9396</v>
       </c>
       <c r="P12" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="Q12" s="45">
+      <c r="Q12" s="43">
         <v>6.9599999999999995E-2</v>
       </c>
       <c r="R12" s="29">
@@ -1112,19 +1459,19 @@
       <c r="C13" s="27">
         <v>0.04</v>
       </c>
-      <c r="D13" s="41">
+      <c r="D13" s="39">
         <f t="shared" si="0"/>
         <v>120000</v>
       </c>
-      <c r="E13" s="41">
+      <c r="E13" s="39">
         <f t="shared" si="1"/>
         <v>112000</v>
       </c>
-      <c r="F13" s="41">
+      <c r="F13" s="39">
         <f t="shared" si="2"/>
         <v>140000</v>
       </c>
-      <c r="G13" s="41">
+      <c r="G13" s="39">
         <f t="shared" si="3"/>
         <v>72000</v>
       </c>
@@ -1151,22 +1498,22 @@
       <c r="B14" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="C14" s="43">
+      <c r="C14" s="41">
         <v>0.02</v>
       </c>
-      <c r="D14" s="41">
+      <c r="D14" s="39">
         <f t="shared" si="0"/>
         <v>60000</v>
       </c>
-      <c r="E14" s="41">
+      <c r="E14" s="39">
         <f t="shared" si="1"/>
         <v>56000</v>
       </c>
-      <c r="F14" s="41">
+      <c r="F14" s="39">
         <f t="shared" si="2"/>
         <v>70000</v>
       </c>
-      <c r="G14" s="41">
+      <c r="G14" s="39">
         <f t="shared" si="3"/>
         <v>36000</v>
       </c>
@@ -1193,22 +1540,22 @@
       <c r="B15" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="C15" s="43">
+      <c r="C15" s="41">
         <v>0.03</v>
       </c>
-      <c r="D15" s="41">
+      <c r="D15" s="39">
         <f t="shared" si="0"/>
         <v>90000</v>
       </c>
-      <c r="E15" s="41">
+      <c r="E15" s="39">
         <f t="shared" si="1"/>
         <v>84000</v>
       </c>
-      <c r="F15" s="41">
+      <c r="F15" s="39">
         <f t="shared" si="2"/>
         <v>105000</v>
       </c>
-      <c r="G15" s="41">
+      <c r="G15" s="39">
         <f t="shared" si="3"/>
         <v>54000</v>
       </c>
@@ -1235,29 +1582,29 @@
       <c r="B16" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="C16" s="47">
+      <c r="C16" s="45">
         <v>8.3299999999999999E-2</v>
       </c>
-      <c r="D16" s="41">
+      <c r="D16" s="39">
         <f>E$3*C16</f>
         <v>249900</v>
       </c>
-      <c r="E16" s="41">
+      <c r="E16" s="39">
         <f t="shared" si="1"/>
         <v>233240</v>
       </c>
-      <c r="F16" s="41">
+      <c r="F16" s="39">
         <f t="shared" si="2"/>
         <v>291550</v>
       </c>
-      <c r="G16" s="41">
+      <c r="G16" s="39">
         <f t="shared" si="3"/>
         <v>149940</v>
       </c>
       <c r="P16" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="Q16" s="40">
+      <c r="Q16" s="38">
         <v>8.3299999999999999E-2</v>
       </c>
       <c r="R16" s="28">
@@ -1277,29 +1624,29 @@
       <c r="B17" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="C17" s="44">
+      <c r="C17" s="42">
         <v>8.3299999999999999E-2</v>
       </c>
-      <c r="D17" s="41">
+      <c r="D17" s="39">
         <f t="shared" si="0"/>
         <v>249900</v>
       </c>
-      <c r="E17" s="41">
+      <c r="E17" s="39">
         <f t="shared" si="1"/>
         <v>233240</v>
       </c>
-      <c r="F17" s="41">
+      <c r="F17" s="39">
         <f t="shared" si="2"/>
         <v>291550</v>
       </c>
-      <c r="G17" s="41">
+      <c r="G17" s="39">
         <f t="shared" si="3"/>
         <v>149940</v>
       </c>
       <c r="P17" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="Q17" s="40">
+      <c r="Q17" s="38">
         <v>8.3299999999999999E-2</v>
       </c>
       <c r="R17" s="28">
@@ -1319,22 +1666,22 @@
       <c r="B18" s="22" t="s">
         <v>44</v>
       </c>
-      <c r="C18" s="43">
+      <c r="C18" s="41">
         <v>0.01</v>
       </c>
-      <c r="D18" s="41">
+      <c r="D18" s="39">
         <f t="shared" si="0"/>
         <v>30000</v>
       </c>
-      <c r="E18" s="41">
+      <c r="E18" s="39">
         <f t="shared" si="1"/>
         <v>28000</v>
       </c>
-      <c r="F18" s="41">
+      <c r="F18" s="39">
         <f t="shared" si="2"/>
         <v>35000</v>
       </c>
-      <c r="G18" s="41">
+      <c r="G18" s="39">
         <f t="shared" si="3"/>
         <v>18000</v>
       </c>
@@ -1361,29 +1708,29 @@
       <c r="B19" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="C19" s="44">
+      <c r="C19" s="42">
         <v>4.1700000000000001E-2</v>
       </c>
-      <c r="D19" s="41">
+      <c r="D19" s="39">
         <f t="shared" si="0"/>
         <v>125100</v>
       </c>
-      <c r="E19" s="41">
+      <c r="E19" s="39">
         <f t="shared" si="1"/>
         <v>116760</v>
       </c>
-      <c r="F19" s="41">
+      <c r="F19" s="39">
         <f t="shared" si="2"/>
         <v>145950</v>
       </c>
-      <c r="G19" s="41">
+      <c r="G19" s="39">
         <f t="shared" si="3"/>
         <v>75060</v>
       </c>
       <c r="P19" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="Q19" s="40">
+      <c r="Q19" s="38">
         <v>4.1700000000000001E-2</v>
       </c>
       <c r="R19" s="28">
@@ -1403,27 +1750,27 @@
       <c r="B20" s="23" t="s">
         <v>45</v>
       </c>
-      <c r="C20" s="44"/>
-      <c r="D20" s="41">
+      <c r="C20" s="42"/>
+      <c r="D20" s="39">
         <f>SUM(D10:D19)</f>
         <v>1555560</v>
       </c>
-      <c r="E20" s="41">
-        <f t="shared" ref="E20:G20" si="4">SUM(E10:E19)</f>
+      <c r="E20" s="39">
+        <f t="shared" ref="E20" si="4">SUM(E10:E19)</f>
         <v>1451856</v>
       </c>
-      <c r="F20" s="41">
+      <c r="F20" s="39">
         <f>SUM(F10+F11+F12+F13+F14+F15+F16+F17+F19+F18)</f>
         <v>1814820</v>
       </c>
-      <c r="G20" s="41">
+      <c r="G20" s="39">
         <f>SUM(G10+G11+G12+G13+G14+G15+G16+G17+G19+G18)</f>
         <v>933336</v>
       </c>
       <c r="P20" s="23" t="s">
         <v>45</v>
       </c>
-      <c r="Q20" s="40">
+      <c r="Q20" s="38">
         <v>0.58289999999999997</v>
       </c>
       <c r="R20" s="28">
@@ -1431,16 +1778,16 @@
       </c>
     </row>
     <row r="23" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B23" s="31" t="s">
+      <c r="B23" s="46" t="s">
         <v>50</v>
       </c>
-      <c r="C23" s="31"/>
-      <c r="D23" s="31"/>
-      <c r="F23" s="31" t="s">
+      <c r="C23" s="46"/>
+      <c r="D23" s="46"/>
+      <c r="F23" s="46" t="s">
         <v>51</v>
       </c>
-      <c r="G23" s="31"/>
-      <c r="H23" s="31"/>
+      <c r="G23" s="46"/>
+      <c r="H23" s="46"/>
     </row>
     <row r="24" spans="2:22" ht="30" x14ac:dyDescent="0.25">
       <c r="B24" s="19" t="s">
@@ -1747,9 +2094,426 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD4EADBE-B4AE-4F9B-87E8-5D2F0560DF26}">
-  <dimension ref="A1"/>
+  <dimension ref="B4:U13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <sheetData>
+    <row r="4" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="C4" s="48" t="s">
+        <v>54</v>
+      </c>
+      <c r="D4" s="48"/>
+      <c r="E4" s="48"/>
+      <c r="F4" s="48"/>
+      <c r="G4" s="48"/>
+      <c r="J4" s="49" t="s">
+        <v>55</v>
+      </c>
+      <c r="K4" s="49"/>
+      <c r="L4" s="49"/>
+      <c r="M4" s="49"/>
+      <c r="N4" s="49"/>
+      <c r="Q4" s="50" t="s">
+        <v>56</v>
+      </c>
+      <c r="R4" s="50"/>
+      <c r="S4" s="50"/>
+      <c r="T4" s="50"/>
+      <c r="U4" s="50"/>
+    </row>
+    <row r="5" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="C5" s="51" t="s">
+        <v>57</v>
+      </c>
+      <c r="D5" s="51" t="s">
+        <v>58</v>
+      </c>
+      <c r="E5" s="52" t="s">
+        <v>59</v>
+      </c>
+      <c r="F5" s="52"/>
+      <c r="G5" s="52"/>
+      <c r="J5" s="53" t="s">
+        <v>57</v>
+      </c>
+      <c r="K5" s="53" t="s">
+        <v>58</v>
+      </c>
+      <c r="L5" s="54" t="s">
+        <v>59</v>
+      </c>
+      <c r="M5" s="54"/>
+      <c r="N5" s="54"/>
+      <c r="Q5" s="55" t="s">
+        <v>57</v>
+      </c>
+      <c r="R5" s="55" t="s">
+        <v>58</v>
+      </c>
+      <c r="S5" s="56" t="s">
+        <v>59</v>
+      </c>
+      <c r="T5" s="56"/>
+      <c r="U5" s="56"/>
+    </row>
+    <row r="6" spans="2:21" ht="30" x14ac:dyDescent="0.25">
+      <c r="B6" s="57" t="s">
+        <v>60</v>
+      </c>
+      <c r="C6" s="26" t="s">
+        <v>61</v>
+      </c>
+      <c r="D6" s="58">
+        <v>1196883</v>
+      </c>
+      <c r="E6" s="59" t="s">
+        <v>62</v>
+      </c>
+      <c r="F6" s="59"/>
+      <c r="G6" s="59"/>
+      <c r="I6" s="60" t="s">
+        <v>60</v>
+      </c>
+      <c r="J6" s="26" t="s">
+        <v>61</v>
+      </c>
+      <c r="K6" s="61">
+        <v>1196883</v>
+      </c>
+      <c r="L6" s="62" t="s">
+        <v>63</v>
+      </c>
+      <c r="M6" s="62"/>
+      <c r="N6" s="62"/>
+      <c r="P6" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q6" s="26" t="s">
+        <v>64</v>
+      </c>
+      <c r="R6" s="63">
+        <v>1213134</v>
+      </c>
+      <c r="S6" s="62" t="s">
+        <v>65</v>
+      </c>
+      <c r="T6" s="62"/>
+      <c r="U6" s="62"/>
+    </row>
+    <row r="7" spans="2:21" ht="75" x14ac:dyDescent="0.25">
+      <c r="B7" s="57" t="s">
+        <v>66</v>
+      </c>
+      <c r="C7" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="D7" s="58">
+        <v>1834000</v>
+      </c>
+      <c r="E7" s="62" t="s">
+        <v>68</v>
+      </c>
+      <c r="F7" s="62"/>
+      <c r="G7" s="62"/>
+      <c r="I7" s="60" t="s">
+        <v>66</v>
+      </c>
+      <c r="J7" s="64" t="s">
+        <v>69</v>
+      </c>
+      <c r="K7" s="26" t="s">
+        <v>69</v>
+      </c>
+      <c r="L7" s="65" t="s">
+        <v>69</v>
+      </c>
+      <c r="M7" s="65"/>
+      <c r="N7" s="65"/>
+      <c r="P7" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q7" s="26" t="s">
+        <v>69</v>
+      </c>
+      <c r="R7" s="26" t="s">
+        <v>69</v>
+      </c>
+      <c r="S7" s="65" t="s">
+        <v>69</v>
+      </c>
+      <c r="T7" s="65"/>
+      <c r="U7" s="65"/>
+    </row>
+    <row r="8" spans="2:21" ht="75" x14ac:dyDescent="0.25">
+      <c r="B8" s="57" t="s">
+        <v>70</v>
+      </c>
+      <c r="C8" s="26" t="s">
+        <v>71</v>
+      </c>
+      <c r="D8" s="61">
+        <v>1600000</v>
+      </c>
+      <c r="E8" s="62" t="s">
+        <v>72</v>
+      </c>
+      <c r="F8" s="62"/>
+      <c r="G8" s="62"/>
+      <c r="I8" s="60" t="s">
+        <v>70</v>
+      </c>
+      <c r="J8" s="26" t="s">
+        <v>73</v>
+      </c>
+      <c r="K8" s="61">
+        <v>1600000</v>
+      </c>
+      <c r="L8" s="62" t="s">
+        <v>74</v>
+      </c>
+      <c r="M8" s="62"/>
+      <c r="N8" s="62"/>
+      <c r="P8" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q8" s="26" t="s">
+        <v>75</v>
+      </c>
+      <c r="R8" s="63">
+        <v>1600000</v>
+      </c>
+      <c r="S8" s="62" t="s">
+        <v>76</v>
+      </c>
+      <c r="T8" s="62"/>
+      <c r="U8" s="62"/>
+    </row>
+    <row r="9" spans="2:21" ht="45" x14ac:dyDescent="0.25">
+      <c r="B9" s="57" t="s">
+        <v>77</v>
+      </c>
+      <c r="C9" s="26" t="s">
+        <v>78</v>
+      </c>
+      <c r="D9" s="61">
+        <v>996959</v>
+      </c>
+      <c r="E9" s="66" t="s">
+        <v>79</v>
+      </c>
+      <c r="F9" s="67"/>
+      <c r="G9" s="68"/>
+      <c r="I9" s="60" t="s">
+        <v>77</v>
+      </c>
+      <c r="J9" s="26" t="s">
+        <v>78</v>
+      </c>
+      <c r="K9" s="61">
+        <v>996959</v>
+      </c>
+      <c r="L9" s="62" t="s">
+        <v>80</v>
+      </c>
+      <c r="M9" s="62"/>
+      <c r="N9" s="62"/>
+      <c r="P9" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="Q9" s="26" t="s">
+        <v>78</v>
+      </c>
+      <c r="R9" s="63">
+        <v>996959</v>
+      </c>
+      <c r="S9" s="62" t="s">
+        <v>81</v>
+      </c>
+      <c r="T9" s="62"/>
+      <c r="U9" s="62"/>
+    </row>
+    <row r="10" spans="2:21" ht="45" x14ac:dyDescent="0.25">
+      <c r="B10" s="57" t="s">
+        <v>82</v>
+      </c>
+      <c r="C10" s="26" t="s">
+        <v>83</v>
+      </c>
+      <c r="D10" s="61">
+        <v>650000</v>
+      </c>
+      <c r="E10" s="62" t="s">
+        <v>84</v>
+      </c>
+      <c r="F10" s="62"/>
+      <c r="G10" s="62"/>
+      <c r="I10" s="60" t="s">
+        <v>82</v>
+      </c>
+      <c r="J10" s="26" t="s">
+        <v>83</v>
+      </c>
+      <c r="K10" s="61">
+        <v>650000</v>
+      </c>
+      <c r="L10" s="62" t="s">
+        <v>85</v>
+      </c>
+      <c r="M10" s="62"/>
+      <c r="N10" s="62"/>
+      <c r="P10" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q10" s="26" t="s">
+        <v>86</v>
+      </c>
+      <c r="R10" s="63">
+        <v>440000</v>
+      </c>
+      <c r="S10" s="62" t="s">
+        <v>87</v>
+      </c>
+      <c r="T10" s="62"/>
+      <c r="U10" s="62"/>
+    </row>
+    <row r="11" spans="2:21" ht="60" x14ac:dyDescent="0.25">
+      <c r="B11" s="57" t="s">
+        <v>88</v>
+      </c>
+      <c r="C11" s="26" t="s">
+        <v>89</v>
+      </c>
+      <c r="D11" s="63">
+        <v>420000</v>
+      </c>
+      <c r="E11" s="62" t="s">
+        <v>90</v>
+      </c>
+      <c r="F11" s="62"/>
+      <c r="G11" s="62"/>
+      <c r="I11" s="60" t="s">
+        <v>88</v>
+      </c>
+      <c r="J11" s="26" t="s">
+        <v>91</v>
+      </c>
+      <c r="K11" s="61">
+        <v>420000</v>
+      </c>
+      <c r="L11" s="62" t="s">
+        <v>92</v>
+      </c>
+      <c r="M11" s="62"/>
+      <c r="N11" s="62"/>
+      <c r="P11" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="Q11" s="26" t="s">
+        <v>93</v>
+      </c>
+      <c r="R11" s="63">
+        <v>425000</v>
+      </c>
+      <c r="S11" s="62" t="s">
+        <v>94</v>
+      </c>
+      <c r="T11" s="62"/>
+      <c r="U11" s="62"/>
+    </row>
+    <row r="12" spans="2:21" ht="45" x14ac:dyDescent="0.25">
+      <c r="B12" s="57" t="s">
+        <v>95</v>
+      </c>
+      <c r="C12" s="26" t="s">
+        <v>96</v>
+      </c>
+      <c r="D12" s="63">
+        <v>185000</v>
+      </c>
+      <c r="E12" s="62" t="s">
+        <v>97</v>
+      </c>
+      <c r="F12" s="62"/>
+      <c r="G12" s="62"/>
+      <c r="I12" s="60" t="s">
+        <v>95</v>
+      </c>
+      <c r="J12" s="26" t="s">
+        <v>98</v>
+      </c>
+      <c r="K12" s="61">
+        <v>185000</v>
+      </c>
+      <c r="L12" s="62" t="s">
+        <v>99</v>
+      </c>
+      <c r="M12" s="62"/>
+      <c r="N12" s="62"/>
+      <c r="P12" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q12" s="26" t="s">
+        <v>98</v>
+      </c>
+      <c r="R12" s="63">
+        <v>185000</v>
+      </c>
+      <c r="S12" s="62" t="s">
+        <v>100</v>
+      </c>
+      <c r="T12" s="62"/>
+      <c r="U12" s="62"/>
+    </row>
+    <row r="13" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="C13" s="69" t="s">
+        <v>101</v>
+      </c>
+      <c r="D13" s="70">
+        <v>6880000</v>
+      </c>
+      <c r="J13" s="60" t="s">
+        <v>101</v>
+      </c>
+      <c r="K13" s="61">
+        <v>5050000</v>
+      </c>
+      <c r="Q13" s="71" t="s">
+        <v>101</v>
+      </c>
+      <c r="R13" s="63">
+        <v>4856000</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="27">
+    <mergeCell ref="E12:G12"/>
+    <mergeCell ref="L12:N12"/>
+    <mergeCell ref="S12:U12"/>
+    <mergeCell ref="E10:G10"/>
+    <mergeCell ref="L10:N10"/>
+    <mergeCell ref="S10:U10"/>
+    <mergeCell ref="E11:G11"/>
+    <mergeCell ref="L11:N11"/>
+    <mergeCell ref="S11:U11"/>
+    <mergeCell ref="E8:G8"/>
+    <mergeCell ref="L8:N8"/>
+    <mergeCell ref="S8:U8"/>
+    <mergeCell ref="E9:G9"/>
+    <mergeCell ref="L9:N9"/>
+    <mergeCell ref="S9:U9"/>
+    <mergeCell ref="E6:G6"/>
+    <mergeCell ref="L6:N6"/>
+    <mergeCell ref="S6:U6"/>
+    <mergeCell ref="E7:G7"/>
+    <mergeCell ref="L7:N7"/>
+    <mergeCell ref="S7:U7"/>
+    <mergeCell ref="C4:G4"/>
+    <mergeCell ref="J4:N4"/>
+    <mergeCell ref="Q4:U4"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="L5:N5"/>
+    <mergeCell ref="S5:U5"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>